<commit_message>
recon-app: update data/RRN_Match_History.xlsx [2026-03-18 04:27 UTC]
</commit_message>
<xml_diff>
--- a/data/RRN_Match_History.xlsx
+++ b/data/RRN_Match_History.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placeholder" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RRN_Match_History" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,6 +434,106 @@
           <t>status</t>
         </is>
       </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>settlement_status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>transaction_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>card_hash_id</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>merchant_name_location</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>is_debit</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>authorization_code</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>system_trace_audit_number</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>RRN</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>auth_ccy</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>payment_reference_number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>effective_auth_amount</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>match_key</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Matched_From</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>as_of_date</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>cleared_using_stripe_date</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>cleared_on_run_date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -441,6 +541,26 @@
           <t>No data yet</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>